<commit_message>
Adicionando colunas de etapa de ensino de cada escola
</commit_message>
<xml_diff>
--- a/CensoEscolarMicrodados2024.xlsx
+++ b/CensoEscolarMicrodados2024.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,46 @@
           <t>IN_EJA_MED</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>IN_INF</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>IN_INF_CRE</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>IN_INF_PRE</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>IN_FUND</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>IN_FUND_AI</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>IN_FUND_AF</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>IN_MED</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>IN_ESP</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -495,6 +535,30 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +590,30 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -553,6 +641,14 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -578,6 +674,14 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -603,6 +707,14 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -628,6 +740,14 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -653,6 +773,14 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -678,6 +806,14 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -703,6 +839,14 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -728,6 +872,14 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -760,6 +912,30 @@
       </c>
       <c r="I12" t="n">
         <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -786,6 +962,14 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -811,6 +995,14 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>